<commit_message>
restart kernel in python and calculate manual intersept and slope
</commit_message>
<xml_diff>
--- a/Excel/005 Simple Linear Regression.xlsx
+++ b/Excel/005 Simple Linear Regression.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24131"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\006 Machine Learning\Excel\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{812AC3F8-265F-4B3A-9C04-DCECA537AD1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -18,9 +24,57 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+  <si>
+    <t>Mencari Slope β</t>
+  </si>
+  <si>
+    <t>Cara Cepat</t>
+  </si>
+  <si>
+    <t>diameter</t>
+  </si>
+  <si>
+    <t>harga</t>
+  </si>
+  <si>
+    <t>Cari Varians X</t>
+  </si>
+  <si>
+    <t>S. itu sama kaya 
+ddof di python</t>
+  </si>
+  <si>
+    <t>Covariance X,Y</t>
+  </si>
+  <si>
+    <t>Slope</t>
+  </si>
+  <si>
+    <t>Cara Manual (Sesuai Rumus)</t>
+  </si>
+  <si>
+    <t>Rata-rata X</t>
+  </si>
+  <si>
+    <t>Rata-rata Y</t>
+  </si>
+  <si>
+    <t>Intercept</t>
+  </si>
+  <si>
+    <t>Rata - Rata Y - (Slope * Rata - Rata X)</t>
+  </si>
+  <si>
+    <t>Mencari Intercept α</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,13 +82,49 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,8 +139,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +441,215 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:J20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="5"/>
+      <c r="G4" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>7</v>
+      </c>
+      <c r="D5" s="1">
+        <f xml:space="preserve"> SLOPE(B5:B9, A5:A9)</f>
+        <v>0.9762931034482758</v>
+      </c>
+      <c r="E5" s="1"/>
+      <c r="G5" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="J5" s="6"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>9</v>
+      </c>
+      <c r="G6" s="1">
+        <f>_xlfn.VAR.S(A5:A9)</f>
+        <v>23.199999999999989</v>
+      </c>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1">
+        <f xml:space="preserve"> _xlfn.COVARIANCE.S(A5:A9, B5:B9)</f>
+        <v>22.65</v>
+      </c>
+      <c r="J6" s="1"/>
+    </row>
+    <row r="7" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>13</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H7" s="4"/>
+      <c r="I7" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7" s="6"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>14</v>
+      </c>
+      <c r="B8">
+        <v>17.5</v>
+      </c>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="1">
+        <f>I6/G6</f>
+        <v>0.97629310344827624</v>
+      </c>
+      <c r="J8" s="1"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>18</v>
+      </c>
+      <c r="B9">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="7"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <f xml:space="preserve"> INTERCEPT(B5:B9, A5:A9)</f>
+        <v>1.9655172413793114</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G16" s="6"/>
+    </row>
+    <row r="17" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D17" s="1">
+        <f xml:space="preserve"> AVERAGE(A5:A9)</f>
+        <v>11.2</v>
+      </c>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1">
+        <f xml:space="preserve"> AVERAGE(B5:B9)</f>
+        <v>12.9</v>
+      </c>
+      <c r="G17" s="1"/>
+    </row>
+    <row r="18" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D18" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+    </row>
+    <row r="19" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D19" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+    </row>
+    <row r="20" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D20" s="1">
+        <f>F17 - (I8 * D17)</f>
+        <v>1.9655172413793078</v>
+      </c>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="D18:G18"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="D20:G20"/>
+    <mergeCell ref="A12:D13"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="G7:H8"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="A1:D2"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G4:J4"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
try prediction model linear
</commit_message>
<xml_diff>
--- a/Excel/005 Simple Linear Regression.xlsx
+++ b/Excel/005 Simple Linear Regression.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\006 Machine Learning\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{812AC3F8-265F-4B3A-9C04-DCECA537AD1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B37E0789-EC9C-4380-8705-A719DAE3FA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Slope &amp; Intercept" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>

<commit_message>
find calculate linear regression using toolkit in excel
</commit_message>
<xml_diff>
--- a/Excel/005 Simple Linear Regression.xlsx
+++ b/Excel/005 Simple Linear Regression.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\006 Machine Learning\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B37E0789-EC9C-4380-8705-A719DAE3FA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6181CA5D-A15E-400C-848F-241CFDFBCA1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Slope &amp; Intercept" sheetId="1" r:id="rId1"/>
+    <sheet name="Data" sheetId="2" r:id="rId2"/>
+    <sheet name="Using Tool" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="50">
   <si>
     <t>Mencari Slope β</t>
   </si>
@@ -68,13 +70,121 @@
   </si>
   <si>
     <t>Mencari Intercept α</t>
+  </si>
+  <si>
+    <t>Diameter (Inch)</t>
+  </si>
+  <si>
+    <t>Harga (Dollar)</t>
+  </si>
+  <si>
+    <t>SUMMARY OUTPUT</t>
+  </si>
+  <si>
+    <t>Regression Statistics</t>
+  </si>
+  <si>
+    <t>Multiple R</t>
+  </si>
+  <si>
+    <t>R Square</t>
+  </si>
+  <si>
+    <t>Adjusted R Square</t>
+  </si>
+  <si>
+    <t>Standard Error</t>
+  </si>
+  <si>
+    <t>Observations</t>
+  </si>
+  <si>
+    <t>ANOVA</t>
+  </si>
+  <si>
+    <t>Regression</t>
+  </si>
+  <si>
+    <t>Residual</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>df</t>
+  </si>
+  <si>
+    <t>SS</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>Significance F</t>
+  </si>
+  <si>
+    <t>Coefficients</t>
+  </si>
+  <si>
+    <t>t Stat</t>
+  </si>
+  <si>
+    <t>P-value</t>
+  </si>
+  <si>
+    <t>Lower 95%</t>
+  </si>
+  <si>
+    <t>Upper 95%</t>
+  </si>
+  <si>
+    <t>Lower 95.0%</t>
+  </si>
+  <si>
+    <t>Upper 95.0%</t>
+  </si>
+  <si>
+    <t>RESIDUAL OUTPUT</t>
+  </si>
+  <si>
+    <t>Observation</t>
+  </si>
+  <si>
+    <t>Predicted Harga (Dollar)</t>
+  </si>
+  <si>
+    <t>Residuals</t>
+  </si>
+  <si>
+    <t>Standard Residuals</t>
+  </si>
+  <si>
+    <t>PROBABILITY OUTPUT</t>
+  </si>
+  <si>
+    <t>Percentile</t>
+  </si>
+  <si>
+    <t>Sum</t>
+  </si>
+  <si>
+    <t>Average</t>
+  </si>
+  <si>
+    <t>Running Total</t>
+  </si>
+  <si>
+    <t>Count</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -106,6 +216,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -127,7 +245,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -135,19 +253,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -156,11 +300,13 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -177,6 +323,725 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Diameter (Inch)  Residual Plot</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Data!$A$2:$A$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Using Tool'!$C$25:$C$29</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>-0.82327586206896619</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.77586206896551779</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.2715517241379306</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.8663793103448274</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-1.5387931034482776</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-7BF8-4B6A-9780-A0A9817E9D4C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1371429487"/>
+        <c:axId val="1371434479"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1371429487"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Diameter (Inch)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1371434479"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1371434479"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Residuals</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1371429487"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Diameter (Inch) Line Fit  Plot</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Harga (Dollar)</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:trendline>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Data!$A$2:$A$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Data!$B$2:$B$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>17.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-D229-4781-9573-DE7796C87EC3}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1381560927"/>
+        <c:axId val="1381554271"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1381560927"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Diameter (Inch)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1381554271"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1381554271"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Harga (Dollar)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1381560927"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Normal Probability Plot</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Using Tool'!$F$25:$F$29</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>90</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Using Tool'!$G$25:$G$29</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>17.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-F9D2-4D58-9763-2016B57AB801}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1381559679"/>
+        <c:axId val="1381554687"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1381559679"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Sample Percentile</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1381554687"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1381554687"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Harga (Dollar)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1381559679"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{71105FE5-6A94-474C-AA10-FCF89C23BEA8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{17960244-0327-429B-A22D-4FB349E84EBB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>22860</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>22860</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2E31FECC-EAE7-482B-9523-92BDD5F27109}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -446,36 +1311,36 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="E4" s="5"/>
-      <c r="G4" s="6" t="s">
+      <c r="E4" s="7"/>
+      <c r="G4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5">
@@ -484,19 +1349,19 @@
       <c r="B5">
         <v>7</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="3">
         <f xml:space="preserve"> SLOPE(B5:B9, A5:A9)</f>
         <v>0.9762931034482758</v>
       </c>
-      <c r="E5" s="1"/>
-      <c r="G5" s="6" t="s">
+      <c r="E5" s="3"/>
+      <c r="G5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6" t="s">
+      <c r="H5" s="2"/>
+      <c r="I5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="6"/>
+      <c r="J5" s="2"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6">
@@ -505,16 +1370,16 @@
       <c r="B6">
         <v>9</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="3">
         <f>_xlfn.VAR.S(A5:A9)</f>
         <v>23.199999999999989</v>
       </c>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1">
+      <c r="H6" s="3"/>
+      <c r="I6" s="3">
         <f xml:space="preserve"> _xlfn.COVARIANCE.S(A5:A9, B5:B9)</f>
         <v>22.65</v>
       </c>
-      <c r="J6" s="1"/>
+      <c r="J6" s="3"/>
     </row>
     <row r="7" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7">
@@ -523,14 +1388,14 @@
       <c r="B7">
         <v>13</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H7" s="4"/>
-      <c r="I7" s="6" t="s">
+      <c r="H7" s="6"/>
+      <c r="I7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J7" s="6"/>
+      <c r="J7" s="2"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8">
@@ -539,13 +1404,13 @@
       <c r="B8">
         <v>17.5</v>
       </c>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="1">
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="3">
         <f>I6/G6</f>
         <v>0.97629310344827624</v>
       </c>
-      <c r="J8" s="1"/>
+      <c r="J8" s="3"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9">
@@ -556,78 +1421,89 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B15" s="7"/>
+      <c r="B15" s="5"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16">
         <f xml:space="preserve"> INTERCEPT(B5:B9, A5:A9)</f>
         <v>1.9655172413793114</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6" t="s">
+      <c r="E16" s="2"/>
+      <c r="F16" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G16" s="6"/>
+      <c r="G16" s="2"/>
     </row>
     <row r="17" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D17" s="1">
+      <c r="D17" s="3">
         <f xml:space="preserve"> AVERAGE(A5:A9)</f>
         <v>11.2</v>
       </c>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1">
+      <c r="E17" s="3"/>
+      <c r="F17" s="3">
         <f xml:space="preserve"> AVERAGE(B5:B9)</f>
         <v>12.9</v>
       </c>
-      <c r="G17" s="1"/>
+      <c r="G17" s="3"/>
     </row>
     <row r="18" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
     </row>
     <row r="19" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
     </row>
     <row r="20" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D20" s="1">
+      <c r="D20" s="3">
         <f>F17 - (I8 * D17)</f>
         <v>1.9655172413793078</v>
       </c>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A1:D2"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G4:J4"/>
+    <mergeCell ref="G7:H8"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="I8:J8"/>
     <mergeCell ref="D18:G18"/>
     <mergeCell ref="D19:G19"/>
     <mergeCell ref="D20:G20"/>
@@ -637,19 +1513,435 @@
     <mergeCell ref="D17:E17"/>
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="F17:G17"/>
-    <mergeCell ref="G7:H8"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="A1:D2"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G4:J4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDBB621C-56E9-4AF7-BCB2-5DE1C0416272}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>8</v>
+      </c>
+      <c r="B3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>14</v>
+      </c>
+      <c r="B5">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>18</v>
+      </c>
+      <c r="B6">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9897C8AC-F52C-4E12-B667-4D84E8E66756}">
+  <dimension ref="A1:I29"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="11"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="8">
+        <v>0.95394003817012007</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="8">
+        <v>0.91000159642401024</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="8">
+        <v>0.88000212856534699</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="8">
+        <v>1.7076147914158122</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" s="10"/>
+      <c r="B11" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="8">
+        <v>1</v>
+      </c>
+      <c r="C12" s="8">
+        <v>88.452155172413782</v>
+      </c>
+      <c r="D12" s="8">
+        <v>88.452155172413782</v>
+      </c>
+      <c r="E12" s="8">
+        <v>30.333924611973401</v>
+      </c>
+      <c r="F12" s="8">
+        <v>1.1784081249034168E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="8">
+        <v>3</v>
+      </c>
+      <c r="C13" s="8">
+        <v>8.7478448275862029</v>
+      </c>
+      <c r="D13" s="8">
+        <v>2.9159482758620676</v>
+      </c>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+    </row>
+    <row r="14" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="9">
+        <v>4</v>
+      </c>
+      <c r="C14" s="9">
+        <v>97.199999999999989</v>
+      </c>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+    </row>
+    <row r="15" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" s="10"/>
+      <c r="B16" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" s="8">
+        <v>1.9655172413793114</v>
+      </c>
+      <c r="C17" s="8">
+        <v>2.1271453463770533</v>
+      </c>
+      <c r="D17" s="8">
+        <v>0.92401642639369874</v>
+      </c>
+      <c r="E17" s="8">
+        <v>0.42362903781866873</v>
+      </c>
+      <c r="F17" s="8">
+        <v>-4.8040086069997772</v>
+      </c>
+      <c r="G17" s="8">
+        <v>8.735043089758399</v>
+      </c>
+      <c r="H17" s="8">
+        <v>-4.8040086069997772</v>
+      </c>
+      <c r="I17" s="8">
+        <v>8.735043089758399</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" s="9">
+        <v>0.9762931034482758</v>
+      </c>
+      <c r="C18" s="9">
+        <v>0.17726211219808774</v>
+      </c>
+      <c r="D18" s="9">
+        <v>5.5076242257413863</v>
+      </c>
+      <c r="E18" s="9">
+        <v>1.1784081249034168E-2</v>
+      </c>
+      <c r="F18" s="9">
+        <v>0.41216594941668516</v>
+      </c>
+      <c r="G18" s="9">
+        <v>1.5404202574798664</v>
+      </c>
+      <c r="H18" s="9">
+        <v>0.41216594941668516</v>
+      </c>
+      <c r="I18" s="9">
+        <v>1.5404202574798664</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>39</v>
+      </c>
+      <c r="F22" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="G24" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" s="8">
+        <v>1</v>
+      </c>
+      <c r="B25" s="8">
+        <v>7.8232758620689662</v>
+      </c>
+      <c r="C25" s="8">
+        <v>-0.82327586206896619</v>
+      </c>
+      <c r="D25" s="8">
+        <v>-0.55670464202145264</v>
+      </c>
+      <c r="F25" s="8">
+        <v>10</v>
+      </c>
+      <c r="G25" s="8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" s="8">
+        <v>2</v>
+      </c>
+      <c r="B26" s="8">
+        <v>9.7758620689655178</v>
+      </c>
+      <c r="C26" s="8">
+        <v>-0.77586206896551779</v>
+      </c>
+      <c r="D26" s="8">
+        <v>-0.52464311813540032</v>
+      </c>
+      <c r="F26" s="8">
+        <v>30</v>
+      </c>
+      <c r="G26" s="8">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" s="8">
+        <v>3</v>
+      </c>
+      <c r="B27" s="8">
+        <v>11.728448275862069</v>
+      </c>
+      <c r="C27" s="8">
+        <v>1.2715517241379306</v>
+      </c>
+      <c r="D27" s="8">
+        <v>0.85983177694412738</v>
+      </c>
+      <c r="F27" s="8">
+        <v>50</v>
+      </c>
+      <c r="G27" s="8">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" s="8">
+        <v>4</v>
+      </c>
+      <c r="B28" s="8">
+        <v>15.633620689655173</v>
+      </c>
+      <c r="C28" s="8">
+        <v>1.8663793103448274</v>
+      </c>
+      <c r="D28" s="8">
+        <v>1.2620581675146008</v>
+      </c>
+      <c r="F28" s="8">
+        <v>70</v>
+      </c>
+      <c r="G28" s="8">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="9">
+        <v>5</v>
+      </c>
+      <c r="B29" s="9">
+        <v>19.538793103448278</v>
+      </c>
+      <c r="C29" s="9">
+        <v>-1.5387931034482776</v>
+      </c>
+      <c r="D29" s="9">
+        <v>-1.0405421843018776</v>
+      </c>
+      <c r="F29" s="9">
+        <v>90</v>
+      </c>
+      <c r="G29" s="9">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G25:G29">
+    <sortCondition ref="G25"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>